<commit_message>
docs(data_dictionary/3.5-special-material-handling): 添加 fxn-wms 全域数据字典文档; 添加 3.5 特殊物料入库流程；
新增完整的数据库模型文档，涵盖 WMS (SQL Server) 和 WES (PostgreSQL) 的完整数据字典，
包括业务主数据、执行数据、审计日志及系统降级支持模型，详细描述了各个表结构和字段定义。
</commit_message>
<xml_diff>
--- a/docs/功能归属表.xlsx
+++ b/docs/功能归属表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaizhou/SynologyDrive/works/fxn-wms/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{021A3CB8-5265-1949-A2FE-17D021B2CA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD03C9D9-E451-EF4A-973A-E5DE49DEE5BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="21240" xr2:uid="{83DC34A4-855E-F341-94CD-123EDADA1840}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="153">
   <si>
     <t>功能模块</t>
   </si>
@@ -399,6 +399,106 @@
   </si>
   <si>
     <t>✅ 接收任务</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>QMS 职责</t>
+  </si>
+  <si>
+    <t>PDA 职责</t>
+  </si>
+  <si>
+    <t>物料分类识别</t>
+  </si>
+  <si>
+    <t>✅ 读取物料主数据</t>
+  </si>
+  <si>
+    <t>路由决策</t>
+  </si>
+  <si>
+    <t>✅ 根据物料类型决策路径</t>
+  </si>
+  <si>
+    <t>库位分配</t>
+  </si>
+  <si>
+    <t>✅ 自动分配目标库位</t>
+  </si>
+  <si>
+    <t>码头绑定</t>
+  </si>
+  <si>
+    <t>✅ 记录绑定关系</t>
+  </si>
+  <si>
+    <t>✅ 扫码绑定</t>
+  </si>
+  <si>
+    <t>运输调度</t>
+  </si>
+  <si>
+    <t>✅ 调用 RCS API</t>
+  </si>
+  <si>
+    <t>IQC 取样</t>
+  </si>
+  <si>
+    <t>✅ 生成取样任务</t>
+  </si>
+  <si>
+    <t>✅ 接收取样请求</t>
+  </si>
+  <si>
+    <t>✅ 扫码取样</t>
+  </si>
+  <si>
+    <t>检验结果处理</t>
+  </si>
+  <si>
+    <t>✅ 接收并处理检验结果</t>
+  </si>
+  <si>
+    <t>✅ 推送检验结果</t>
+  </si>
+  <si>
+    <t>入库确认</t>
+  </si>
+  <si>
+    <t>✅ 更新库存状态</t>
+  </si>
+  <si>
+    <t>✅ 扫码确认</t>
+  </si>
+  <si>
+    <t>六合一绑定</t>
+  </si>
+  <si>
+    <t>手动扫描送货</t>
+  </si>
+  <si>
+    <t>✅ 生成运输任务</t>
+  </si>
+  <si>
+    <t>✅ 扫码操作</t>
+  </si>
+  <si>
+    <t>库存管理</t>
+  </si>
+  <si>
+    <t>✅ 维护库存数据</t>
+  </si>
+  <si>
+    <t>✅ 人工操作</t>
+  </si>
+  <si>
+    <t>SAP 同步</t>
+  </si>
+  <si>
+    <t>✅ 批量同步库存数据</t>
+  </si>
+  <si>
+    <t>特殊物料入库</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -845,7 +945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{945DC6DF-BE66-CF42-AA2D-016BA392A074}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="22" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20" style="2" bestFit="1" customWidth="1"/>
@@ -1852,6 +1952,256 @@
         <v>8</v>
       </c>
     </row>
+    <row r="56" spans="1:6" ht="22" customHeight="1">
+      <c r="A56" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+    </row>
+    <row r="57" spans="1:6" ht="22" customHeight="1">
+      <c r="A57" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="22" customHeight="1">
+      <c r="A58" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="22" customHeight="1">
+      <c r="A59" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="22" customHeight="1">
+      <c r="A60" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="22" customHeight="1">
+      <c r="A61" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="22" customHeight="1">
+      <c r="A62" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F62" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="22" customHeight="1">
+      <c r="A63" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F63" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="22" customHeight="1">
+      <c r="A64" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F64" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="22" customHeight="1">
+      <c r="A65" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="22" customHeight="1">
+      <c r="A66" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="22" customHeight="1">
+      <c r="A67" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F67" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="22" customHeight="1">
+      <c r="A68" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="22" customHeight="1">
+      <c r="A69" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="22" customHeight="1">
+      <c r="A70" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>